<commit_message>
0.55: Fachreferat über die Spalte der Personenliste, UPL trägt das Fachreferat ein, mehr Abstand
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/UPL_Vorlage.xlsx
+++ b/bedarfsliste-app/UPL_Vorlage.xlsx
@@ -124,7 +124,7 @@
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="60" customWidth="1"/>
     <col min="9" max="9" width="40" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="34" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
@@ -182,7 +182,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dienst</t>
+          <t xml:space="preserve">Fachreferat</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -6115,12 +6115,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dienst</t>
+          <t xml:space="preserve">Fachreferat</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aus „Dienst“, unverändert (z. B. KATS, SAND, AU).</t>
+          <t xml:space="preserve">Das Fachreferat, zu dem der Bedarf gehört (in der UPL in der Spalte „Dienst“), z. B. Notfallvorsorge oder Soziales Ehrenamt – genau so geschrieben wie in der Personenliste in der Spalte „Fachreferat“; darüber ordnet die Bedarfsliste die Ansprechpersonen des Fachreferats zu. Steht in der UPL nur ein Kürzel (z. B. KATS, SAND) und ist das Fachreferat nicht eindeutig: Kürzel übernehmen und in „Hinweis“ vermerken.</t>
         </is>
       </c>
     </row>

</xml_diff>